<commit_message>
ci: fix deploy workflow + actualizar Excel y cache-bust
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist_qn90g8e\OneDrive\Documentos\Desarrollo Vs Code\.vscode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist_qn90g8e\OneDrive\Documentos\Desarrollo Vs Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9933630-6F57-453E-BA1D-4097D76936F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF8AE0B-ECA2-4C47-AABE-30FCC33543F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,44 +22,6 @@
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>ChatGPT</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Formato: YYYY-MM-DD</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Formato: YYYY-MM-DD</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -896,7 +858,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2416,7 +2378,9 @@
       <c r="D66" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E66" s="3"/>
+      <c r="E66" s="3">
+        <v>45962</v>
+      </c>
       <c r="F66" s="2" t="s">
         <v>78</v>
       </c>
@@ -2437,7 +2401,9 @@
       <c r="D67" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E67" s="3"/>
+      <c r="E67" s="3">
+        <v>45962</v>
+      </c>
       <c r="F67" s="2" t="s">
         <v>78</v>
       </c>
@@ -2458,7 +2424,9 @@
       <c r="D68" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E68" s="3"/>
+      <c r="E68" s="3">
+        <v>45962</v>
+      </c>
       <c r="F68" s="2" t="s">
         <v>78</v>
       </c>
@@ -2479,7 +2447,9 @@
       <c r="D69" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E69" s="3"/>
+      <c r="E69" s="3">
+        <v>45962</v>
+      </c>
       <c r="F69" s="2" t="s">
         <v>78</v>
       </c>
@@ -2500,7 +2470,9 @@
       <c r="D70" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E70" s="3"/>
+      <c r="E70" s="3">
+        <v>45962</v>
+      </c>
       <c r="F70" s="2" t="s">
         <v>78</v>
       </c>
@@ -2521,7 +2493,9 @@
       <c r="D71" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E71" s="3"/>
+      <c r="E71" s="3">
+        <v>45962</v>
+      </c>
       <c r="F71" s="2" t="s">
         <v>78</v>
       </c>
@@ -2542,7 +2516,9 @@
       <c r="D72" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E72" s="3"/>
+      <c r="E72" s="3">
+        <v>45962</v>
+      </c>
       <c r="F72" s="2" t="s">
         <v>78</v>
       </c>
@@ -2553,7 +2529,6 @@
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">

</xml_diff>

<commit_message>
republicar dashboard en GitHub Pages
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -8,24 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist_qn90g8e\OneDrive\Documentos\Desarrollo Vs Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF8AE0B-ECA2-4C47-AABE-30FCC33543F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BA2FA5-31C6-4E8F-A22A-EA88C1133A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
-    <sheet name="Listas" sheetId="2" r:id="rId2"/>
-    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
+    <sheet name="Enlaces" sheetId="4" r:id="rId2"/>
+    <sheet name="Listas" sheetId="2" r:id="rId3"/>
+    <sheet name="Instrucciones" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="160">
   <si>
     <t>Implementación</t>
   </si>
@@ -219,9 +220,6 @@
     <t>Onboarding</t>
   </si>
   <si>
-    <t>Entrega maqueta inducción corporativa</t>
-  </si>
-  <si>
     <t>Iniciado en plazo</t>
   </si>
   <si>
@@ -285,12 +283,6 @@
     <t>Propuesta financiera</t>
   </si>
   <si>
-    <t>Entrega maqueta cultura servicio</t>
-  </si>
-  <si>
-    <t>Entrega diseño final inducción corporativa</t>
-  </si>
-  <si>
     <t>Jorge.García</t>
   </si>
   <si>
@@ -330,12 +322,6 @@
     <t>Kick Off Champions</t>
   </si>
   <si>
-    <t>Entrega maqueta habilitación colaboradores</t>
-  </si>
-  <si>
-    <t>Entrega diseño final cultura servicio</t>
-  </si>
-  <si>
     <t>Ejecución de formación</t>
   </si>
   <si>
@@ -354,24 +340,12 @@
     <t>Kick off cultura Data-Driven</t>
   </si>
   <si>
-    <t>Entrega maqueta competencias y funciones propias del rol</t>
-  </si>
-  <si>
-    <t>Entrega diseño final habilitación colaboradores</t>
-  </si>
-  <si>
     <t>Entrega de informe</t>
   </si>
   <si>
     <t>Desarrollar mapa</t>
   </si>
   <si>
-    <t>Entrega maqueta champion técnico mucamas</t>
-  </si>
-  <si>
-    <t>Entrega diseño final competencias y funciones propias del rol</t>
-  </si>
-  <si>
     <t>Diseño del modelo de organización por área: manual del rol champions</t>
   </si>
   <si>
@@ -387,12 +361,6 @@
     <t>Formación de Embajadores RRHH y Logística: Entrenamiento y certificación de sus equipos</t>
   </si>
   <si>
-    <t>Entrega final material inducción</t>
-  </si>
-  <si>
-    <t>Entrega final material cultura</t>
-  </si>
-  <si>
     <t>Entrega diseño final champion técnico mucamas</t>
   </si>
   <si>
@@ -466,13 +434,85 @@
   </si>
   <si>
     <t>Owner</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Nobel%20Biocare</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Ópticas%20Schilling</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Promet</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Cromtek</t>
+  </si>
+  <si>
+    <t>Imilfex</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Imilfex</t>
+  </si>
+  <si>
+    <t>Check Persons / Komatsu</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Check%20Persons%20Komatsu</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=Cementos%20Melón</t>
+  </si>
+  <si>
+    <t>🔗 https://cristobalalfaro-cmd.github.io/dashboard-proyectos/?cliente=BioNet</t>
+  </si>
+  <si>
+    <t>Construcción maqueta versión resumida</t>
+  </si>
+  <si>
+    <t>Desarrollo contenidos inducción hotelería</t>
+  </si>
+  <si>
+    <t>Desarrollo contenidos Cultura de Servicio</t>
+  </si>
+  <si>
+    <t>Desarrollo contenidos Habilitación Colaboradores</t>
+  </si>
+  <si>
+    <t>Desarrollo contenidos Rol de Mucama</t>
+  </si>
+  <si>
+    <t>Validación coontenidos</t>
+  </si>
+  <si>
+    <t>Encargados de Hotel</t>
+  </si>
+  <si>
+    <t>Cristóbal Alfaro</t>
+  </si>
+  <si>
+    <t>Construcción versión final (mas resumida, no tan extensa, más práctica)</t>
+  </si>
+  <si>
+    <t>Jorge García (Sprint)</t>
+  </si>
+  <si>
+    <t>Diseño gráfico presentaciones (todos los módulos)</t>
+  </si>
+  <si>
+    <t>Diseño Manual del Participante (Inducción)</t>
+  </si>
+  <si>
+    <t>Diseño Manual del Participante (Mucama)</t>
+  </si>
+  <si>
+    <t>Diseño Manual de Coaching para "Champion" (Mucama)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -485,6 +525,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -506,7 +554,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -544,17 +592,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -859,41 +920,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G72"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="7" width="14" customWidth="1"/>
+    <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="68.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
@@ -916,7 +979,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -939,7 +1002,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
@@ -962,7 +1025,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
@@ -985,7 +1048,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -1008,7 +1071,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
@@ -1031,7 +1094,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>30</v>
       </c>
@@ -1054,7 +1117,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -1077,7 +1140,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -1100,7 +1163,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>30</v>
       </c>
@@ -1123,7 +1186,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>59</v>
       </c>
@@ -1146,7 +1209,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>59</v>
       </c>
@@ -1180,30 +1243,30 @@
         <v>63</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>64</v>
+        <v>147</v>
       </c>
       <c r="E14" s="3">
         <v>45929</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="E15" s="3">
         <v>45931</v>
@@ -1215,18 +1278,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E16" s="3">
         <v>45932</v>
@@ -1238,7 +1301,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>59</v>
       </c>
@@ -1246,10 +1309,10 @@
         <v>2</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="E17" s="3">
         <v>45933</v>
@@ -1261,53 +1324,53 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="E18" s="3">
         <v>45933</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="E19" s="3">
         <v>45933</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>59</v>
       </c>
@@ -1318,19 +1381,19 @@
         <v>60</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E20" s="3">
         <v>45933</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G20" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>59</v>
       </c>
@@ -1338,22 +1401,22 @@
         <v>5</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="E21" s="3">
         <v>45933</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>59</v>
       </c>
@@ -1361,22 +1424,22 @@
         <v>5</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E22" s="3">
         <v>45933</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>59</v>
       </c>
@@ -1384,39 +1447,39 @@
         <v>5</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E23" s="3">
         <v>45933</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E24" s="3">
         <v>45936</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>35</v>
@@ -1433,16 +1496,16 @@
         <v>63</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="E25" s="3">
         <v>45936</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1455,66 +1518,66 @@
       <c r="C26" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>87</v>
+      <c r="D26" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="E26" s="3">
         <v>45936</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E27" s="3">
         <v>45940</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="E28" s="3">
         <v>45940</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>59</v>
       </c>
@@ -1522,22 +1585,22 @@
         <v>5</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E29" s="3">
         <v>45940</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>59</v>
       </c>
@@ -1545,22 +1608,22 @@
         <v>5</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E30" s="3">
         <v>45940</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>59</v>
       </c>
@@ -1568,22 +1631,22 @@
         <v>2</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E31" s="3">
         <v>45940</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>59</v>
       </c>
@@ -1591,45 +1654,45 @@
         <v>2</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E32" s="3">
         <v>45940</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E33" s="3">
         <v>45937</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>59</v>
       </c>
@@ -1637,16 +1700,16 @@
         <v>2</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E34" s="3">
         <v>45943</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>35</v>
@@ -1663,16 +1726,16 @@
         <v>63</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>101</v>
+        <v>150</v>
       </c>
       <c r="E35" s="3">
         <v>45943</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -1686,88 +1749,88 @@
         <v>63</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>102</v>
+        <v>151</v>
       </c>
       <c r="E36" s="3">
-        <v>45943</v>
+        <v>45936</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E37" s="3">
         <v>45947</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E38" s="3">
         <v>45947</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E39" s="3">
         <v>45947</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>59</v>
       </c>
@@ -1775,22 +1838,22 @@
         <v>5</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E40" s="3">
         <v>45947</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>59</v>
       </c>
@@ -1798,22 +1861,22 @@
         <v>5</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E41" s="3">
         <v>45947</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>59</v>
       </c>
@@ -1821,16 +1884,16 @@
         <v>2</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E42" s="3">
         <v>45950</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>35</v>
@@ -1847,16 +1910,16 @@
         <v>63</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="E43" s="3">
-        <v>45950</v>
+        <v>45943</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -1870,42 +1933,42 @@
         <v>63</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="E44" s="3">
         <v>45950</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E45" s="3">
         <v>45954</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>59</v>
       </c>
@@ -1913,16 +1976,16 @@
         <v>5</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E46" s="3">
         <v>45954</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>35</v>
@@ -1939,16 +2002,16 @@
         <v>63</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>113</v>
+        <v>156</v>
       </c>
       <c r="E47" s="3">
         <v>45957</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>35</v>
+        <v>155</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
@@ -1962,19 +2025,19 @@
         <v>63</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>114</v>
+        <v>157</v>
       </c>
       <c r="E48" s="3">
         <v>45957</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>59</v>
       </c>
@@ -1982,22 +2045,22 @@
         <v>2</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="E49" s="3">
         <v>45961</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>59</v>
       </c>
@@ -2005,22 +2068,22 @@
         <v>2</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="E50" s="3">
         <v>45961</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>59</v>
       </c>
@@ -2028,22 +2091,22 @@
         <v>2</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E51" s="3">
         <v>45961</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>59</v>
       </c>
@@ -2051,22 +2114,22 @@
         <v>2</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E52" s="3">
         <v>45964</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>59</v>
       </c>
@@ -2074,16 +2137,16 @@
         <v>2</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="E53" s="3">
         <v>45964</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>35</v>
@@ -2100,16 +2163,16 @@
         <v>63</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="E54" s="3">
         <v>45964</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
@@ -2123,16 +2186,16 @@
         <v>63</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>121</v>
+        <v>159</v>
       </c>
       <c r="E55" s="3">
         <v>45964</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
@@ -2146,19 +2209,19 @@
         <v>63</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="E56" s="3">
         <v>45964</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>59</v>
       </c>
@@ -2166,22 +2229,22 @@
         <v>5</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="E57" s="3">
         <v>45968</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>59</v>
       </c>
@@ -2189,22 +2252,22 @@
         <v>2</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E58" s="3">
         <v>45971</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>59</v>
       </c>
@@ -2212,16 +2275,16 @@
         <v>2</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="E59" s="3">
         <v>45971</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>35</v>
@@ -2238,16 +2301,16 @@
         <v>63</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="E60" s="3">
         <v>45971</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
@@ -2261,19 +2324,19 @@
         <v>63</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="E61" s="3">
         <v>45971</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>59</v>
       </c>
@@ -2281,22 +2344,22 @@
         <v>5</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="E62" s="3">
         <v>45975</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>59</v>
       </c>
@@ -2304,22 +2367,22 @@
         <v>5</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="E63" s="3">
         <v>45982</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>59</v>
       </c>
@@ -2327,45 +2390,45 @@
         <v>5</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="E64" s="3">
         <v>45989</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="E65" s="3">
         <v>45943</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>59</v>
       </c>
@@ -2373,22 +2436,22 @@
         <v>2</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="E66" s="3">
         <v>45962</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>59</v>
       </c>
@@ -2396,22 +2459,22 @@
         <v>2</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="E67" s="3">
         <v>45962</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G67" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>59</v>
       </c>
@@ -2419,22 +2482,22 @@
         <v>2</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="E68" s="3">
         <v>45962</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G68" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>59</v>
       </c>
@@ -2442,22 +2505,22 @@
         <v>2</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="E69" s="3">
         <v>45962</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G69" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>59</v>
       </c>
@@ -2465,22 +2528,22 @@
         <v>2</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="E70" s="3">
         <v>45962</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G70" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>59</v>
       </c>
@@ -2488,22 +2551,22 @@
         <v>2</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="E71" s="3">
         <v>45962</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G71" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>59</v>
       </c>
@@ -2511,23 +2574,34 @@
         <v>2</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="E72" s="3">
         <v>45962</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>35</v>
       </c>
     </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D75" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G72" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Promet"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2551,9 +2625,106 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189A26BC-CE5E-41B9-AD1E-6F9B5F4CF130}">
+  <dimension ref="A1:A23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="87.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -2597,7 +2768,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Agrego data.json y actualizo template
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist_qn90g8e\OneDrive\Documentos\Desarrollo Vs Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45D5501F-813C-4A27-A53A-511D8F0A7096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7C4ADB-36CB-4957-92FC-03BE5383831C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1180,7 +1180,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -1433,7 +1433,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
@@ -1456,7 +1456,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>32</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
@@ -1663,7 +1663,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>32</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>32</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>32</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>32</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>32</v>
       </c>
@@ -1962,7 +1962,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>32</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>32</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>32</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>32</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
         <v>32</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>32</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="8" t="s">
         <v>32</v>
       </c>
@@ -2608,25 +2608,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G75" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="6">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Loreto.Naranjo"/>
+        <filter val="Promet"/>
       </filters>
     </filterColumn>
   </autoFilter>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="E76:E994" xr:uid="{00000000-0002-0000-0000-000001000000}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>E76:E994</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
auto: publish 08-10-2025 17:56:41,92
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d2dcec49e3bc7bf/Documentos/Desarrollo Vs Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3CA5977-4951-4A93-8F63-70F38DEF678C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="132">
   <si>
     <t>Ópticas Schilling</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Finalizado</t>
   </si>
   <si>
-    <t>Cristobal.Alfaro</t>
-  </si>
-  <si>
     <t>Sprint/Starbuks</t>
   </si>
   <si>
@@ -179,9 +176,6 @@
     <t>On hold</t>
   </si>
   <si>
-    <t>Nicolás.Araya</t>
-  </si>
-  <si>
     <t>E-Learning CST</t>
   </si>
   <si>
@@ -191,9 +185,6 @@
     <t>Desarrollo caso 1</t>
   </si>
   <si>
-    <t>Jorge.Cadiz</t>
-  </si>
-  <si>
     <t>Desarrollar evaluación módulo 1</t>
   </si>
   <si>
@@ -230,9 +221,6 @@
     <t>Licitación modelo gestión instructores</t>
   </si>
   <si>
-    <t>Loreto.Naranjo</t>
-  </si>
-  <si>
     <t>Kick Off Champions</t>
   </si>
   <si>
@@ -423,6 +411,15 @@
   </si>
   <si>
     <t>Reunión de traspaso (habilitación) presentaciones a Encargados de Personas de cada Hotel</t>
+  </si>
+  <si>
+    <t>Jorge Cádiz</t>
+  </si>
+  <si>
+    <t>Loreto Naranjo</t>
+  </si>
+  <si>
+    <t>Nicolás Araya</t>
   </si>
 </sst>
 </file>
@@ -841,7 +838,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -856,28 +852,28 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -897,21 +893,21 @@
         <v>7</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="E3" s="3">
         <v>45915</v>
@@ -920,21 +916,21 @@
         <v>7</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="E4" s="3">
         <v>45915</v>
@@ -943,21 +939,21 @@
         <v>7</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="E5" s="3">
         <v>45915</v>
@@ -966,21 +962,21 @@
         <v>7</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="E6" s="3">
         <v>45915</v>
@@ -989,21 +985,21 @@
         <v>7</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" s="3">
         <v>45915</v>
@@ -1012,21 +1008,21 @@
         <v>7</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="3">
         <v>45915</v>
@@ -1035,21 +1031,21 @@
         <v>7</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="3">
         <v>45915</v>
@@ -1058,21 +1054,21 @@
         <v>7</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="E10" s="3">
         <v>45915</v>
@@ -1081,21 +1077,21 @@
         <v>7</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="E11" s="3">
         <v>45915</v>
@@ -1104,21 +1100,21 @@
         <v>7</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="E12" s="3">
         <v>45923</v>
@@ -1127,21 +1123,21 @@
         <v>7</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E13" s="3">
         <v>45923</v>
@@ -1150,21 +1146,21 @@
         <v>7</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E14" s="3">
         <v>45929</v>
@@ -1173,21 +1169,21 @@
         <v>7</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="E15" s="3">
         <v>45931</v>
@@ -1196,21 +1192,21 @@
         <v>7</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E16" s="3">
         <v>45932</v>
@@ -1219,21 +1215,21 @@
         <v>7</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="E17" s="3">
         <v>45933</v>
@@ -1242,182 +1238,182 @@
         <v>7</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="E18" s="3">
         <v>45933</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="E19" s="3">
         <v>45933</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E20" s="3">
         <v>45933</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E21" s="3">
         <v>45933</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="E22" s="3">
         <v>45933</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E23" s="3">
         <v>45933</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E24" s="3">
         <v>45936</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E25" s="3">
         <v>45936</v>
@@ -1426,21 +1422,21 @@
         <v>7</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E26" s="3">
         <v>45936</v>
@@ -1449,228 +1445,228 @@
         <v>7</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E27" s="3">
         <v>45940</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="E28" s="3">
         <v>45940</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E29" s="3">
         <v>45940</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E30" s="3">
         <v>45940</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E31" s="3">
         <v>45940</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E32" s="3">
         <v>45940</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E33" s="3">
         <v>45937</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E34" s="3">
         <v>45943</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E35" s="3">
         <v>45943</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E36" s="3">
         <v>45936</v>
@@ -1679,868 +1675,862 @@
         <v>7</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E37" s="3">
         <v>45947</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E38" s="3">
         <v>45947</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E39" s="3">
         <v>45947</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E40" s="3">
         <v>45947</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E41" s="3">
         <v>45947</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E42" s="3">
         <v>45950</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E43" s="3">
         <v>45943</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E44" s="3">
         <v>45950</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E45" s="3">
         <v>45954</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E46" s="3">
         <v>45954</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E47" s="3">
         <v>45957</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E48" s="3">
         <v>45964</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E49" s="3">
         <v>45961</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E50" s="3">
         <v>45961</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E51" s="3">
         <v>45961</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E52" s="3">
         <v>45964</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E53" s="3">
         <v>45964</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E54" s="3">
         <v>45964</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E55" s="3">
         <v>45964</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E56" s="3">
         <v>45971</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E57" s="3">
         <v>45968</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E58" s="3">
         <v>45971</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E59" s="3">
         <v>45971</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E60" s="3">
         <v>45978</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E61" s="3">
         <v>45978</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E62" s="3">
         <v>45975</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E63" s="3">
         <v>45982</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E64" s="3">
         <v>45989</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E65" s="3">
         <v>45943</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E66" s="3">
         <v>45962</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E67" s="3">
         <v>45962</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E68" s="3">
         <v>45962</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E69" s="3">
         <v>45962</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E70" s="3">
         <v>45962</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E71" s="3">
         <v>45962</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E72" s="3">
         <v>45962</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E73" s="3">
         <v>45957</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G73" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Promet"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G73" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D74:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>#REF!</formula1>
@@ -2565,7 +2555,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
@@ -2575,7 +2565,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
@@ -2585,57 +2575,57 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: publish 08-10-2025 18:11:37,35
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d2dcec49e3bc7bf/Documentos/Desarrollo Vs Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3CA5977-4951-4A93-8F63-70F38DEF678C}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B02E8F7F-CE24-462D-802D-E6780EE75051}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="137">
   <si>
     <t>Ópticas Schilling</t>
   </si>
@@ -155,9 +155,6 @@
     <t>Data Lake</t>
   </si>
   <si>
-    <t>Entrega PPT Kick off Data Driven</t>
-  </si>
-  <si>
     <t>Cromtek</t>
   </si>
   <si>
@@ -212,18 +209,9 @@
     <t>Desarrollar evaluación módulo 2</t>
   </si>
   <si>
-    <t>Revisión Data Lake (RRHH y logística)</t>
-  </si>
-  <si>
-    <t>Diseño PPTT Kick off Champions</t>
-  </si>
-  <si>
     <t>Licitación modelo gestión instructores</t>
   </si>
   <si>
-    <t>Kick Off Champions</t>
-  </si>
-  <si>
     <t>Ejecución de formación</t>
   </si>
   <si>
@@ -239,9 +227,6 @@
     <t>Desarrollar evaluación módulo 3</t>
   </si>
   <si>
-    <t>Kick off cultura Data-Driven</t>
-  </si>
-  <si>
     <t>Entrega de informe</t>
   </si>
   <si>
@@ -420,6 +405,36 @@
   </si>
   <si>
     <t>Nicolás Araya</t>
+  </si>
+  <si>
+    <t>Desarrollo PPT Kick off Data Driven</t>
+  </si>
+  <si>
+    <t>Acceso Data Lake (RRHH y logística)</t>
+  </si>
+  <si>
+    <t>Atrasado</t>
+  </si>
+  <si>
+    <t>Osvaldo Muñoz</t>
+  </si>
+  <si>
+    <t>Reunión Kick Off Champions</t>
+  </si>
+  <si>
+    <t>Reunión Kick off cultura Data-Driven</t>
+  </si>
+  <si>
+    <t>Validación PPT Kick off Champions</t>
+  </si>
+  <si>
+    <t>Entrega diseño PPT Kick off Champions</t>
+  </si>
+  <si>
+    <t>Marcela y Osvaldo</t>
+  </si>
+  <si>
+    <t>Validación PPT Kick off cultura Data Driven</t>
   </si>
 </sst>
 </file>
@@ -838,7 +853,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G73"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
@@ -852,28 +868,28 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -893,10 +909,10 @@
         <v>7</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -916,10 +932,10 @@
         <v>7</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -939,10 +955,10 @@
         <v>7</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -962,10 +978,10 @@
         <v>7</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -985,10 +1001,10 @@
         <v>7</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -1008,10 +1024,10 @@
         <v>7</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -1031,10 +1047,10 @@
         <v>7</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1054,10 +1070,10 @@
         <v>7</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -1077,10 +1093,10 @@
         <v>7</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -1100,10 +1116,10 @@
         <v>7</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>31</v>
       </c>
@@ -1123,10 +1139,10 @@
         <v>7</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
@@ -1146,10 +1162,10 @@
         <v>7</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1160,7 +1176,7 @@
         <v>35</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E14" s="3">
         <v>45929</v>
@@ -1169,10 +1185,10 @@
         <v>7</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -1192,10 +1208,10 @@
         <v>7</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>3</v>
       </c>
@@ -1215,7 +1231,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1229,7 +1245,7 @@
         <v>42</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="E17" s="3">
         <v>45933</v>
@@ -1238,56 +1254,56 @@
         <v>7</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E18" s="3">
         <v>45933</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E19" s="3">
         <v>45933</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
@@ -1298,19 +1314,19 @@
         <v>32</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E20" s="3">
         <v>45933</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>31</v>
       </c>
@@ -1318,22 +1334,22 @@
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="E21" s="3">
         <v>45933</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
@@ -1341,10 +1357,10 @@
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E22" s="3">
         <v>45933</v>
@@ -1353,10 +1369,10 @@
         <v>7</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>31</v>
       </c>
@@ -1364,22 +1380,22 @@
         <v>1</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E23" s="3">
         <v>45933</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
@@ -1390,7 +1406,7 @@
         <v>38</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E24" s="3">
         <v>45936</v>
@@ -1399,10 +1415,10 @@
         <v>36</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>31</v>
       </c>
@@ -1413,7 +1429,7 @@
         <v>35</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E25" s="3">
         <v>45936</v>
@@ -1422,10 +1438,10 @@
         <v>7</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>31</v>
       </c>
@@ -1436,7 +1452,7 @@
         <v>35</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E26" s="3">
         <v>45936</v>
@@ -1445,56 +1461,56 @@
         <v>7</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E27" s="3">
         <v>45940</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G27" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="E28" s="3">
         <v>45940</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
@@ -1502,22 +1518,22 @@
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E29" s="3">
         <v>45940</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1525,19 +1541,19 @@
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E30" s="3">
         <v>45940</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -1551,16 +1567,16 @@
         <v>42</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>62</v>
+        <v>128</v>
       </c>
       <c r="E31" s="3">
-        <v>45940</v>
+        <v>45933</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>36</v>
+        <v>129</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
@@ -1574,7 +1590,7 @@
         <v>42</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>63</v>
+        <v>134</v>
       </c>
       <c r="E32" s="3">
         <v>45940</v>
@@ -1583,18 +1599,18 @@
         <v>36</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>39</v>
@@ -1603,10 +1619,10 @@
         <v>45937</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
@@ -1620,19 +1636,19 @@
         <v>42</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="E34" s="3">
         <v>45943</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
@@ -1643,7 +1659,7 @@
         <v>35</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E35" s="3">
         <v>45943</v>
@@ -1652,10 +1668,10 @@
         <v>36</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>31</v>
       </c>
@@ -1666,7 +1682,7 @@
         <v>35</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E36" s="3">
         <v>45936</v>
@@ -1675,79 +1691,79 @@
         <v>7</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E37" s="3">
         <v>45947</v>
       </c>
       <c r="F37" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="D38" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E38" s="3">
         <v>45947</v>
       </c>
       <c r="F38" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="D39" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E39" s="3">
         <v>45947</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>31</v>
       </c>
@@ -1755,22 +1771,22 @@
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E40" s="3">
         <v>45947</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>31</v>
       </c>
@@ -1778,19 +1794,19 @@
         <v>1</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E41" s="3">
         <v>45947</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -1804,19 +1820,19 @@
         <v>42</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>71</v>
+        <v>132</v>
       </c>
       <c r="E42" s="3">
         <v>45950</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>31</v>
       </c>
@@ -1827,7 +1843,7 @@
         <v>35</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E43" s="3">
         <v>45943</v>
@@ -1836,10 +1852,10 @@
         <v>36</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>31</v>
       </c>
@@ -1850,42 +1866,42 @@
         <v>35</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E44" s="3">
         <v>45950</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E45" s="3">
         <v>45954</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>31</v>
       </c>
@@ -1893,22 +1909,22 @@
         <v>1</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E46" s="3">
         <v>45954</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>31</v>
       </c>
@@ -1919,19 +1935,19 @@
         <v>35</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E47" s="3">
         <v>45957</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>31</v>
       </c>
@@ -1942,16 +1958,16 @@
         <v>35</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E48" s="3">
         <v>45964</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
@@ -1965,16 +1981,16 @@
         <v>42</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E49" s="3">
         <v>45961</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -1988,16 +2004,16 @@
         <v>42</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E50" s="3">
         <v>45961</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -2011,16 +2027,16 @@
         <v>42</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E51" s="3">
         <v>45961</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
@@ -2034,16 +2050,16 @@
         <v>42</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E52" s="3">
         <v>45964</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
@@ -2057,19 +2073,19 @@
         <v>42</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E53" s="3">
         <v>45964</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>31</v>
       </c>
@@ -2080,19 +2096,19 @@
         <v>35</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E54" s="3">
         <v>45964</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>31</v>
       </c>
@@ -2103,19 +2119,19 @@
         <v>35</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E55" s="3">
         <v>45964</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>31</v>
       </c>
@@ -2126,19 +2142,19 @@
         <v>35</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E56" s="3">
         <v>45971</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>31</v>
       </c>
@@ -2146,19 +2162,19 @@
         <v>1</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E57" s="3">
         <v>45968</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
@@ -2172,16 +2188,16 @@
         <v>42</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E58" s="3">
         <v>45971</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
@@ -2195,19 +2211,19 @@
         <v>42</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E59" s="3">
         <v>45971</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>31</v>
       </c>
@@ -2218,19 +2234,19 @@
         <v>35</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="E60" s="3">
         <v>45978</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>31</v>
       </c>
@@ -2241,19 +2257,19 @@
         <v>35</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E61" s="3">
         <v>45978</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>31</v>
       </c>
@@ -2261,22 +2277,22 @@
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E62" s="3">
         <v>45975</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>31</v>
       </c>
@@ -2284,22 +2300,22 @@
         <v>1</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E63" s="3">
         <v>45982</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>31</v>
       </c>
@@ -2307,42 +2323,42 @@
         <v>1</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E64" s="3">
         <v>45989</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E65" s="3">
         <v>45943</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
@@ -2356,16 +2372,16 @@
         <v>42</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E66" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
@@ -2379,16 +2395,16 @@
         <v>42</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E67" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
@@ -2402,16 +2418,16 @@
         <v>42</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E68" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
@@ -2425,16 +2441,16 @@
         <v>42</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E69" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
@@ -2448,16 +2464,16 @@
         <v>42</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E70" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
@@ -2471,16 +2487,16 @@
         <v>42</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E71" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
@@ -2494,19 +2510,19 @@
         <v>42</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E72" s="3">
-        <v>45962</v>
+        <v>45976</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>31</v>
       </c>
@@ -2517,22 +2533,74 @@
         <v>35</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E73" s="3">
         <v>45957</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>114</v>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E74" s="3">
+        <v>45943</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E75" s="3">
+        <v>45947</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G73" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G73" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Ópticas Schilling"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D74:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D76:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
@@ -2555,7 +2623,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
@@ -2565,7 +2633,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
@@ -2575,37 +2643,37 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
@@ -2615,7 +2683,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
@@ -2625,7 +2693,7 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: publish 08-10-2025 19:14:21,55
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d2dcec49e3bc7bf/Documentos/Desarrollo Vs Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B02E8F7F-CE24-462D-802D-E6780EE75051}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5000B94-0CC3-46C0-88CF-A483117EACC1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Enlaces" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$H$75</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="140">
   <si>
     <t>Ópticas Schilling</t>
   </si>
@@ -435,13 +435,22 @@
   </si>
   <si>
     <t>Validación PPT Kick off cultura Data Driven</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>cristobal.alfaro.s@outlook.com</t>
+  </si>
+  <si>
+    <t>Loreto.naranjo@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -459,6 +468,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -483,7 +500,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -532,11 +549,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF263143"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF263143"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF263143"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -549,8 +593,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -854,7 +908,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
@@ -866,7 +920,7 @@
     <col min="7" max="7" width="17.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
@@ -885,11 +939,14 @@
       <c r="F1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="8" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H1" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -908,11 +965,14 @@
       <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -931,11 +991,14 @@
       <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -954,11 +1017,14 @@
       <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -977,11 +1043,14 @@
       <c r="F5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1000,11 +1069,14 @@
       <c r="F6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G6" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -1023,11 +1095,14 @@
       <c r="F7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G7" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -1046,11 +1121,14 @@
       <c r="F8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1069,11 +1147,14 @@
       <c r="F9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G9" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -1092,11 +1173,14 @@
       <c r="F10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G10" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -1115,11 +1199,14 @@
       <c r="F11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G11" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>31</v>
       </c>
@@ -1138,11 +1225,14 @@
       <c r="F12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G12" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
@@ -1161,11 +1251,14 @@
       <c r="F13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G13" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1184,11 +1277,14 @@
       <c r="F14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G14" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -1207,11 +1303,14 @@
       <c r="F15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G15" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>3</v>
       </c>
@@ -1230,11 +1329,14 @@
       <c r="F16" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G16" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -1253,11 +1355,14 @@
       <c r="F17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G17" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
@@ -1276,11 +1381,14 @@
       <c r="F18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G18" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
@@ -1299,11 +1407,14 @@
       <c r="F19" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G19" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
@@ -1322,11 +1433,14 @@
       <c r="F20" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="9" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H20" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>31</v>
       </c>
@@ -1345,11 +1459,14 @@
       <c r="F21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G21" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G21" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
@@ -1368,11 +1485,14 @@
       <c r="F22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" s="9" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>31</v>
       </c>
@@ -1391,11 +1511,14 @@
       <c r="F23" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G23" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
@@ -1414,11 +1537,14 @@
       <c r="F24" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G24" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G24" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>31</v>
       </c>
@@ -1437,11 +1563,14 @@
       <c r="F25" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G25" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G25" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>31</v>
       </c>
@@ -1460,11 +1589,14 @@
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G26" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G26" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>31</v>
       </c>
@@ -1483,11 +1615,14 @@
       <c r="F27" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G27" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G27" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>31</v>
       </c>
@@ -1506,11 +1641,14 @@
       <c r="F28" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G28" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G28" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
@@ -1529,11 +1667,14 @@
       <c r="F29" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="G29" s="9" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H29" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1552,11 +1693,14 @@
       <c r="F30" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G30" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G30" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
@@ -1575,11 +1719,14 @@
       <c r="F31" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="9" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H31" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
@@ -1598,11 +1745,14 @@
       <c r="F32" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G32" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G32" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
@@ -1621,11 +1771,14 @@
       <c r="F33" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="10" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H33" s="12" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>31</v>
       </c>
@@ -1644,11 +1797,14 @@
       <c r="F34" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G34" s="9" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H34" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
@@ -1667,11 +1823,14 @@
       <c r="F35" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G35" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G35" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>31</v>
       </c>
@@ -1690,11 +1849,14 @@
       <c r="F36" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="G36" s="9" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H36" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -1713,11 +1875,14 @@
       <c r="F37" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G37" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
@@ -1736,11 +1901,14 @@
       <c r="F38" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G38" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>31</v>
       </c>
@@ -1759,11 +1927,14 @@
       <c r="F39" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G39" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G39" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>31</v>
       </c>
@@ -1782,11 +1953,14 @@
       <c r="F40" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G40" s="3" t="s">
+      <c r="G40" s="9" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H40" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>31</v>
       </c>
@@ -1805,11 +1979,14 @@
       <c r="F41" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G41" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G41" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H41" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>31</v>
       </c>
@@ -1828,11 +2005,14 @@
       <c r="F42" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G42" s="3" t="s">
+      <c r="G42" s="9" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H42" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>31</v>
       </c>
@@ -1851,11 +2031,14 @@
       <c r="F43" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G43" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G43" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>31</v>
       </c>
@@ -1874,11 +2057,14 @@
       <c r="F44" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G44" s="3" t="s">
+      <c r="G44" s="9" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H44" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
@@ -1897,11 +2083,14 @@
       <c r="F45" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G45" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G45" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H45" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>31</v>
       </c>
@@ -1920,11 +2109,14 @@
       <c r="F46" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G46" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G46" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H46" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>31</v>
       </c>
@@ -1943,11 +2135,14 @@
       <c r="F47" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G47" s="3" t="s">
+      <c r="G47" s="9" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H47" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>31</v>
       </c>
@@ -1966,11 +2161,14 @@
       <c r="F48" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G48" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G48" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H48" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>31</v>
       </c>
@@ -1989,11 +2187,14 @@
       <c r="F49" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G49" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G49" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H49" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>31</v>
       </c>
@@ -2012,11 +2213,14 @@
       <c r="F50" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G50" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G50" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>31</v>
       </c>
@@ -2035,11 +2239,14 @@
       <c r="F51" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G51" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G51" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>31</v>
       </c>
@@ -2058,11 +2265,14 @@
       <c r="F52" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G52" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G52" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H52" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>31</v>
       </c>
@@ -2081,11 +2291,14 @@
       <c r="F53" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G53" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G53" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H53" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>31</v>
       </c>
@@ -2104,11 +2317,14 @@
       <c r="F54" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G54" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G54" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H54" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>31</v>
       </c>
@@ -2127,11 +2343,14 @@
       <c r="F55" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G55" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G55" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H55" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>31</v>
       </c>
@@ -2150,11 +2369,14 @@
       <c r="F56" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G56" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G56" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H56" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>31</v>
       </c>
@@ -2173,11 +2395,14 @@
       <c r="F57" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G57" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G57" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H57" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>31</v>
       </c>
@@ -2196,11 +2421,14 @@
       <c r="F58" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G58" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G58" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H58" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>31</v>
       </c>
@@ -2219,11 +2447,14 @@
       <c r="F59" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G59" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G59" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H59" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>31</v>
       </c>
@@ -2242,11 +2473,14 @@
       <c r="F60" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G60" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G60" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H60" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>31</v>
       </c>
@@ -2265,11 +2499,14 @@
       <c r="F61" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G61" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G61" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H61" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>31</v>
       </c>
@@ -2288,11 +2525,14 @@
       <c r="F62" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G62" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G62" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H62" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>31</v>
       </c>
@@ -2311,11 +2551,14 @@
       <c r="F63" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G63" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G63" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H63" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>31</v>
       </c>
@@ -2334,11 +2577,14 @@
       <c r="F64" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G64" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G64" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H64" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>3</v>
       </c>
@@ -2357,11 +2603,14 @@
       <c r="F65" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G65" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G65" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H65" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>31</v>
       </c>
@@ -2380,11 +2629,14 @@
       <c r="F66" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G66" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G66" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H66" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>31</v>
       </c>
@@ -2403,11 +2655,14 @@
       <c r="F67" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G67" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G67" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H67" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>31</v>
       </c>
@@ -2426,11 +2681,14 @@
       <c r="F68" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G68" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G68" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H68" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>31</v>
       </c>
@@ -2449,11 +2707,14 @@
       <c r="F69" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G69" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G69" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H69" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>31</v>
       </c>
@@ -2472,11 +2733,14 @@
       <c r="F70" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G70" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G70" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H70" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>31</v>
       </c>
@@ -2495,11 +2759,14 @@
       <c r="F71" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G71" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G71" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H71" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>31</v>
       </c>
@@ -2518,11 +2785,14 @@
       <c r="F72" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G72" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G72" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H72" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>31</v>
       </c>
@@ -2541,11 +2811,14 @@
       <c r="F73" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G73" s="3" t="s">
+      <c r="G73" s="9" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H73" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>31</v>
       </c>
@@ -2564,11 +2837,14 @@
       <c r="F74" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G74" s="3" t="s">
+      <c r="G74" s="9" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H74" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>31</v>
       </c>
@@ -2587,15 +2863,18 @@
       <c r="F75" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G75" s="3" t="s">
+      <c r="G75" s="9" t="s">
         <v>135</v>
       </c>
+      <c r="H75" s="12" t="s">
+        <v>138</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G73" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
+  <autoFilter ref="A1:H75" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="6">
       <filters>
-        <filter val="Ópticas Schilling"/>
+        <filter val="Loreto Naranjo"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2604,6 +2883,9 @@
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H33" r:id="rId1" xr:uid="{532945AD-3F8A-412E-B67E-D681483A4EF7}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
auto: publish 09-10-2025 15:01:02,78
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -5,26 +5,39 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d2dcec49e3bc7bf/Documentos/Desarrollo Vs Code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist_qn90g8e\OneDrive\Documentos\Desarrollo Vs Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="8_{A947079A-5E47-44B2-B312-EF9329BCD015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5000B94-0CC3-46C0-88CF-A483117EACC1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10AE3003-B25B-432A-8DC0-2C8C68ACC5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4680" yWindow="-16320" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
     <sheet name="Enlaces" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$H$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$H$76</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="144">
   <si>
     <t>Ópticas Schilling</t>
   </si>
@@ -365,9 +378,6 @@
     <t>Jorge García (Sprint)</t>
   </si>
   <si>
-    <t>Diseño gráfico presentaciones (todos los módulos)</t>
-  </si>
-  <si>
     <t>Reunión de traspaso (habilitación) manual Aux. Aseo a Encargados de Personas y Jefes de ese rol</t>
   </si>
   <si>
@@ -377,9 +387,6 @@
     <t>Revisión de contenidos</t>
   </si>
   <si>
-    <t>Validación contenidos + agregar info propia de cada hotel</t>
-  </si>
-  <si>
     <t>Desarrollo contenidos Rol de Aux. Aseo / Mucama</t>
   </si>
   <si>
@@ -444,6 +451,24 @@
   </si>
   <si>
     <t>Loreto.naranjo@gmail.com</t>
+  </si>
+  <si>
+    <t>jgarcia@sprint.cl</t>
+  </si>
+  <si>
+    <t>Diseño Gráfico Kick Off General y Kick off para los Champions</t>
+  </si>
+  <si>
+    <t>Validación contenidos + agregar info propia de cada hotel por parte de los Encargados de Personas de cada Hotel</t>
+  </si>
+  <si>
+    <t>dromo@promet.cl</t>
+  </si>
+  <si>
+    <t>Daniela Romo</t>
+  </si>
+  <si>
+    <t>Diseño gráfico presentacion inducción completa (todos los módulos)</t>
   </si>
 </sst>
 </file>
@@ -908,16 +933,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="85.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="99.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.77734375" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -943,7 +969,7 @@
         <v>95</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -969,7 +995,7 @@
         <v>110</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -995,7 +1021,7 @@
         <v>110</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1021,7 +1047,7 @@
         <v>110</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1047,7 +1073,7 @@
         <v>110</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1073,7 +1099,7 @@
         <v>110</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1099,7 +1125,7 @@
         <v>110</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1125,7 +1151,7 @@
         <v>110</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1151,7 +1177,7 @@
         <v>110</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1177,7 +1203,7 @@
         <v>110</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1203,7 +1229,7 @@
         <v>110</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1229,7 +1255,7 @@
         <v>110</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1255,10 +1281,10 @@
         <v>110</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1281,7 +1307,7 @@
         <v>110</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1307,7 +1333,7 @@
         <v>110</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1333,7 +1359,7 @@
         <v>110</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1347,7 +1373,7 @@
         <v>42</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E17" s="3">
         <v>45933</v>
@@ -1359,7 +1385,7 @@
         <v>110</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1385,7 +1411,7 @@
         <v>110</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1411,7 +1437,7 @@
         <v>110</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1434,10 +1460,10 @@
         <v>48</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1463,7 +1489,7 @@
         <v>110</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1486,10 +1512,10 @@
         <v>7</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1515,7 +1541,7 @@
         <v>110</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1541,10 +1567,10 @@
         <v>110</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>31</v>
       </c>
@@ -1567,10 +1593,10 @@
         <v>110</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>31</v>
       </c>
@@ -1593,7 +1619,7 @@
         <v>110</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1619,7 +1645,7 @@
         <v>110</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1645,7 +1671,7 @@
         <v>110</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1668,10 +1694,10 @@
         <v>55</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1697,7 +1723,7 @@
         <v>110</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1711,19 +1737,19 @@
         <v>42</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E31" s="3">
         <v>45933</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1737,7 +1763,7 @@
         <v>42</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E32" s="3">
         <v>45940</v>
@@ -1749,10 +1775,10 @@
         <v>110</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
@@ -1772,10 +1798,10 @@
         <v>55</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1789,7 +1815,7 @@
         <v>42</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E34" s="3">
         <v>45943</v>
@@ -1798,13 +1824,13 @@
         <v>55</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>31</v>
       </c>
@@ -1815,7 +1841,7 @@
         <v>35</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E35" s="3">
         <v>45943</v>
@@ -1827,10 +1853,10 @@
         <v>110</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>31</v>
       </c>
@@ -1841,7 +1867,7 @@
         <v>35</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E36" s="3">
         <v>45936</v>
@@ -1853,7 +1879,7 @@
         <v>109</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1879,7 +1905,7 @@
         <v>110</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1905,7 +1931,7 @@
         <v>110</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1931,7 +1957,7 @@
         <v>110</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1954,10 +1980,10 @@
         <v>55</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1983,7 +2009,7 @@
         <v>110</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -1997,7 +2023,7 @@
         <v>42</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E42" s="3">
         <v>45950</v>
@@ -2006,13 +2032,13 @@
         <v>55</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>31</v>
       </c>
@@ -2035,10 +2061,10 @@
         <v>110</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>31</v>
       </c>
@@ -2049,7 +2075,7 @@
         <v>35</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="E44" s="3">
         <v>45950</v>
@@ -2061,7 +2087,7 @@
         <v>109</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2087,7 +2113,7 @@
         <v>110</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2113,10 +2139,10 @@
         <v>110</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>31</v>
       </c>
@@ -2127,7 +2153,7 @@
         <v>35</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="E47" s="3">
         <v>45957</v>
@@ -2142,7 +2168,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>31</v>
       </c>
@@ -2153,7 +2179,7 @@
         <v>35</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E48" s="3">
         <v>45964</v>
@@ -2165,7 +2191,7 @@
         <v>110</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2191,7 +2217,7 @@
         <v>110</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2217,7 +2243,7 @@
         <v>110</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2243,7 +2269,7 @@
         <v>110</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2269,7 +2295,7 @@
         <v>110</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2295,10 +2321,10 @@
         <v>110</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>31</v>
       </c>
@@ -2309,7 +2335,7 @@
         <v>35</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E54" s="3">
         <v>45964</v>
@@ -2321,10 +2347,10 @@
         <v>110</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>31</v>
       </c>
@@ -2335,7 +2361,7 @@
         <v>35</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E55" s="3">
         <v>45964</v>
@@ -2347,10 +2373,10 @@
         <v>110</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>31</v>
       </c>
@@ -2361,7 +2387,7 @@
         <v>35</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E56" s="3">
         <v>45971</v>
@@ -2373,7 +2399,7 @@
         <v>110</v>
       </c>
       <c r="H56" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2399,7 +2425,7 @@
         <v>110</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2425,7 +2451,7 @@
         <v>110</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2451,10 +2477,10 @@
         <v>110</v>
       </c>
       <c r="H59" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>31</v>
       </c>
@@ -2465,7 +2491,7 @@
         <v>35</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E60" s="3">
         <v>45978</v>
@@ -2477,10 +2503,10 @@
         <v>110</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>31</v>
       </c>
@@ -2491,7 +2517,7 @@
         <v>35</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E61" s="3">
         <v>45978</v>
@@ -2500,10 +2526,10 @@
         <v>55</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>110</v>
+        <v>142</v>
       </c>
       <c r="H61" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2529,7 +2555,7 @@
         <v>110</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2555,7 +2581,7 @@
         <v>110</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2581,7 +2607,7 @@
         <v>110</v>
       </c>
       <c r="H64" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2607,7 +2633,7 @@
         <v>110</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2633,7 +2659,7 @@
         <v>110</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2659,7 +2685,7 @@
         <v>110</v>
       </c>
       <c r="H67" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2685,7 +2711,7 @@
         <v>110</v>
       </c>
       <c r="H68" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2711,7 +2737,7 @@
         <v>110</v>
       </c>
       <c r="H69" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2737,7 +2763,7 @@
         <v>110</v>
       </c>
       <c r="H70" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2763,7 +2789,7 @@
         <v>110</v>
       </c>
       <c r="H71" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2789,10 +2815,10 @@
         <v>110</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>31</v>
       </c>
@@ -2803,7 +2829,7 @@
         <v>35</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E73" s="3">
         <v>45957</v>
@@ -2815,7 +2841,7 @@
         <v>109</v>
       </c>
       <c r="H73" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2829,7 +2855,7 @@
         <v>42</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E74" s="3">
         <v>45943</v>
@@ -2838,10 +2864,10 @@
         <v>55</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
@@ -2855,7 +2881,7 @@
         <v>42</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E75" s="3">
         <v>45947</v>
@@ -2864,27 +2890,54 @@
         <v>55</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H75" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E76" s="3">
+        <v>45943</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G76" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H76" s="12" t="s">
         <v>138</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H75" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="6">
+  <autoFilter ref="A1:H76" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Loreto Naranjo"/>
+        <filter val="Promet"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D76:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D77:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="H33" r:id="rId1" xr:uid="{532945AD-3F8A-412E-B67E-D681483A4EF7}"/>
+    <hyperlink ref="H47" r:id="rId2" xr:uid="{7C20C5C3-5F88-4C82-8420-B55ECBFEC86E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: publish 10-10-2025 17:21:43,91
</commit_message>
<xml_diff>
--- a/Template_Proyectos_Dashboard.xlsx
+++ b/Template_Proyectos_Dashboard.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist_qn90g8e\OneDrive\Documentos\Desarrollo Vs Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10AE3003-B25B-432A-8DC0-2C8C68ACC5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37E47570-92C9-41A9-9095-B81815293FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4680" yWindow="-16320" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5130" yWindow="-16320" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyectos" sheetId="1" r:id="rId1"/>
     <sheet name="Enlaces" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$H$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyectos!$A$1:$H$80</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="157">
   <si>
     <t>Ópticas Schilling</t>
   </si>
@@ -469,6 +469,45 @@
   </si>
   <si>
     <t>Diseño gráfico presentacion inducción completa (todos los módulos)</t>
+  </si>
+  <si>
+    <t>Reunión 14 de Octubre (Levantamiento)</t>
+  </si>
+  <si>
+    <t>Iniciado</t>
+  </si>
+  <si>
+    <t>Seguimiento propuesta</t>
+  </si>
+  <si>
+    <t>Seguimiento</t>
+  </si>
+  <si>
+    <t>Presentación propuesta</t>
+  </si>
+  <si>
+    <t>Smart Mining</t>
+  </si>
+  <si>
+    <t>Headhunting Full Stack</t>
+  </si>
+  <si>
+    <t>Reclutamiento</t>
+  </si>
+  <si>
+    <t>Entrevistas</t>
+  </si>
+  <si>
+    <t>Envío de candidatos</t>
+  </si>
+  <si>
+    <t>Entrevistas con cliente</t>
+  </si>
+  <si>
+    <t>Evaluación psicolaboral</t>
+  </si>
+  <si>
+    <t>Cierre y facturación</t>
   </si>
 </sst>
 </file>
@@ -932,8 +971,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
@@ -972,7 +1010,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -998,7 +1036,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1024,7 +1062,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1050,7 +1088,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1076,7 +1114,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1102,7 +1140,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -1128,7 +1166,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -1154,7 +1192,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1180,7 +1218,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -1206,7 +1244,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -1232,7 +1270,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>31</v>
       </c>
@@ -1258,7 +1296,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
@@ -1301,7 +1339,7 @@
         <v>45929</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>110</v>
@@ -1310,12 +1348,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>38</v>
@@ -1336,7 +1374,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>3</v>
       </c>
@@ -1362,7 +1400,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -1376,10 +1414,10 @@
         <v>125</v>
       </c>
       <c r="E17" s="3">
-        <v>45933</v>
+        <v>45945</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>110</v>
@@ -1388,7 +1426,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
@@ -1414,7 +1452,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
@@ -1440,7 +1478,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
@@ -1466,7 +1504,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>31</v>
       </c>
@@ -1492,7 +1530,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
@@ -1518,7 +1556,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>31</v>
       </c>
@@ -1544,12 +1582,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>38</v>
@@ -1561,7 +1599,7 @@
         <v>45936</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>110</v>
@@ -1587,7 +1625,7 @@
         <v>45936</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>110</v>
@@ -1613,7 +1651,7 @@
         <v>45936</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>110</v>
@@ -1622,7 +1660,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>31</v>
       </c>
@@ -1648,7 +1686,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>31</v>
       </c>
@@ -1674,7 +1712,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
@@ -1700,7 +1738,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1726,7 +1764,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>31</v>
       </c>
@@ -1752,7 +1790,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
@@ -1778,7 +1816,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
@@ -1795,7 +1833,7 @@
         <v>45937</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>123</v>
@@ -1804,7 +1842,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>31</v>
       </c>
@@ -1818,7 +1856,7 @@
         <v>129</v>
       </c>
       <c r="E34" s="3">
-        <v>45943</v>
+        <v>45946</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>55</v>
@@ -1873,7 +1911,7 @@
         <v>45936</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>109</v>
@@ -1882,7 +1920,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
@@ -1908,7 +1946,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
@@ -1934,7 +1972,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>31</v>
       </c>
@@ -1960,7 +1998,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>31</v>
       </c>
@@ -1986,7 +2024,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>31</v>
       </c>
@@ -2012,7 +2050,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>31</v>
       </c>
@@ -2090,7 +2128,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
@@ -2116,7 +2154,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>31</v>
       </c>
@@ -2194,7 +2232,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>31</v>
       </c>
@@ -2220,7 +2258,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>31</v>
       </c>
@@ -2246,7 +2284,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>31</v>
       </c>
@@ -2272,7 +2310,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>31</v>
       </c>
@@ -2298,7 +2336,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>31</v>
       </c>
@@ -2402,7 +2440,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>31</v>
       </c>
@@ -2428,7 +2466,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>31</v>
       </c>
@@ -2454,7 +2492,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>31</v>
       </c>
@@ -2532,7 +2570,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>31</v>
       </c>
@@ -2558,7 +2596,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>31</v>
       </c>
@@ -2584,7 +2622,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>31</v>
       </c>
@@ -2610,7 +2648,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>3</v>
       </c>
@@ -2636,7 +2674,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>31</v>
       </c>
@@ -2662,7 +2700,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>31</v>
       </c>
@@ -2688,7 +2726,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>31</v>
       </c>
@@ -2714,7 +2752,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>31</v>
       </c>
@@ -2740,7 +2778,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>31</v>
       </c>
@@ -2766,7 +2804,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>31</v>
       </c>
@@ -2792,7 +2830,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>31</v>
       </c>
@@ -2844,7 +2882,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>31</v>
       </c>
@@ -2870,7 +2908,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>31</v>
       </c>
@@ -2896,7 +2934,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>31</v>
       </c>
@@ -2913,7 +2951,7 @@
         <v>45943</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>55</v>
+        <v>145</v>
       </c>
       <c r="G76" s="9" t="s">
         <v>112</v>
@@ -2922,22 +2960,283 @@
         <v>138</v>
       </c>
     </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E77" s="3">
+        <v>45944</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H77" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E78" s="3">
+        <v>45947</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G78" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H78" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A79" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E79" s="3">
+        <v>45947</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H79" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A80" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E80" s="3">
+        <v>45950</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G80" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H80" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E81" s="3">
+        <v>45944</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G81" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H81" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E82" s="3">
+        <v>45947</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G82" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H82" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A83" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E83" s="3">
+        <v>45950</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G83" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H83" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A84" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E84" s="3">
+        <v>45957</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G84" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H84" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A85" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E85" s="3">
+        <v>45960</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G85" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H85" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A86" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E86" s="3">
+        <v>45975</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G86" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H86" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H76" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Promet"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H80" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D77:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="D87:E994" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="H33" r:id="rId1" xr:uid="{532945AD-3F8A-412E-B67E-D681483A4EF7}"/>
     <hyperlink ref="H47" r:id="rId2" xr:uid="{7C20C5C3-5F88-4C82-8420-B55ECBFEC86E}"/>
+    <hyperlink ref="H78" r:id="rId3" xr:uid="{5C3F69FB-BD6B-4A91-9324-180B4453197A}"/>
+    <hyperlink ref="H81" r:id="rId4" xr:uid="{37049263-48B6-4D3F-8EB8-AADBC37EB8F4}"/>
+    <hyperlink ref="H82" r:id="rId5" xr:uid="{C787D3C9-5B3A-47EC-A103-4C822A858D64}"/>
+    <hyperlink ref="H83" r:id="rId6" xr:uid="{43F856F4-B8AB-46CC-A494-990BDA1BC64B}"/>
+    <hyperlink ref="H84" r:id="rId7" xr:uid="{EAC5C8FE-63F6-4A48-8430-BE480141D333}"/>
+    <hyperlink ref="H85" r:id="rId8" xr:uid="{9AC961BA-A489-49BB-825B-B9FB81437931}"/>
+    <hyperlink ref="H86" r:id="rId9" xr:uid="{4C7B1D8A-7815-4040-8EAC-80016F0612E9}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>